<commit_message>
Add Study 2 material and data
</commit_message>
<xml_diff>
--- a/3_simulators/data/ttj_raw_data_variables_explained.xlsx
+++ b/3_simulators/data/ttj_raw_data_variables_explained.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\Github_Mannheim\lnt\simulators\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\Github_Mannheim\time_to_jump\3_simulators\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1EBC1D-39A9-4A13-A1C9-48219E6C85AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB0704E-7F4B-435B-9889-0417A95763D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="s1_letter_number_discrimination" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -596,13 +596,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="75.6640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="75.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -610,7 +610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -618,7 +618,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -626,7 +626,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -634,7 +634,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -642,7 +642,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -658,7 +658,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -666,7 +666,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -674,7 +674,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -682,7 +682,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -690,7 +690,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -698,7 +698,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -706,7 +706,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -714,7 +714,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
@@ -722,7 +722,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
@@ -730,7 +730,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
@@ -738,7 +738,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -746,7 +746,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
@@ -754,7 +754,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -762,7 +762,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>70</v>
       </c>
@@ -770,7 +770,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
@@ -778,7 +778,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>40</v>
       </c>
@@ -786,7 +786,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
@@ -794,23 +794,23 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
@@ -818,7 +818,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
@@ -826,7 +826,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>50</v>
       </c>
@@ -834,7 +834,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>52</v>
       </c>
@@ -842,7 +842,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>54</v>
       </c>
@@ -850,7 +850,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>56</v>
       </c>
@@ -858,7 +858,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>58</v>
       </c>
@@ -866,7 +866,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>60</v>
       </c>
@@ -874,7 +874,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>62</v>
       </c>
@@ -882,7 +882,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>64</v>
       </c>

</xml_diff>